<commit_message>
correcao relatorio de exportação
</commit_message>
<xml_diff>
--- a/relatorio/despesas.xlsx
+++ b/relatorio/despesas.xlsx
@@ -139,7 +139,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -157,6 +157,9 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
@@ -391,332 +394,332 @@
   <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="11.53515625" defaultRowHeight="17.35" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
-    <col width="37.34" customWidth="1" style="6" min="1" max="1"/>
-    <col width="18.36" customWidth="1" style="6" min="2" max="2"/>
-    <col width="32.24" customWidth="1" style="6" min="3" max="3"/>
-    <col width="11.43" customWidth="1" style="7" min="4" max="4"/>
-    <col width="11.53" customWidth="1" style="6" min="5" max="16384"/>
+    <col width="37.34" customWidth="1" style="7" min="1" max="1"/>
+    <col width="18.36" customWidth="1" style="7" min="2" max="2"/>
+    <col width="32.24" customWidth="1" style="7" min="3" max="3"/>
+    <col width="11.43" customWidth="1" style="8" min="4" max="4"/>
+    <col width="11.53" customWidth="1" style="7" min="5" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.35" customHeight="1" s="8">
-      <c r="A1" s="9" t="inlineStr">
+    <row r="1" ht="17.35" customHeight="1" s="9">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Relatório de Despesas de Viagem</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
-      <c r="D1" s="11" t="n"/>
-    </row>
-    <row r="2" ht="14.45" customHeight="1" s="8">
-      <c r="A2" s="9" t="inlineStr">
+      <c r="B1" s="11" t="n"/>
+      <c r="C1" s="11" t="n"/>
+      <c r="D1" s="12" t="n"/>
+    </row>
+    <row r="2" ht="14.45" customHeight="1" s="9">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Empresa: Smart Picking Soluções Digitais Ltda</t>
         </is>
       </c>
-      <c r="B2" s="11" t="n"/>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="B2" s="12" t="n"/>
+      <c r="C2" s="10" t="inlineStr">
         <is>
           <t>Setor: Smart</t>
         </is>
       </c>
-      <c r="D2" s="11" t="n"/>
-    </row>
-    <row r="3" ht="14.45" customHeight="1" s="8">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="D2" s="12" t="n"/>
+    </row>
+    <row r="3" ht="14.45" customHeight="1" s="9">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Colaborador: Fernando Pereira da Trindade</t>
         </is>
       </c>
-      <c r="B3" s="11" t="n"/>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="B3" s="12" t="n"/>
+      <c r="C3" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Retorno: </t>
         </is>
       </c>
-      <c r="D3" s="11" t="n"/>
-    </row>
-    <row r="4" ht="14.45" customHeight="1" s="8">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="D3" s="12" t="n"/>
+    </row>
+    <row r="4" ht="14.45" customHeight="1" s="9">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Destino: Contagem - MG</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="10" t="inlineStr">
         <is>
           <t>Motivo Viagem: Implantação DRL Parte 2</t>
         </is>
       </c>
-      <c r="C4" s="10" t="n"/>
-      <c r="D4" s="11" t="n"/>
-    </row>
-    <row r="5" ht="17.35" customHeight="1" s="8">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="C4" s="11" t="n"/>
+      <c r="D4" s="12" t="n"/>
+    </row>
+    <row r="5" ht="17.35" customHeight="1" s="9">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Saída: Apucarana</t>
         </is>
       </c>
-      <c r="B5" s="9" t="n"/>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="11" t="n"/>
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="12" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n"/>
-      <c r="B6" s="12" t="n"/>
-      <c r="C6" s="12" t="n"/>
-      <c r="D6" s="12" t="n"/>
-    </row>
-    <row r="7" ht="17.35" customHeight="1" s="8">
-      <c r="A7" s="9" t="inlineStr">
+      <c r="A6" s="13" t="n"/>
+      <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="17.35" customHeight="1" s="9">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Descrição Das Despesas</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="10" t="n"/>
-      <c r="D7" s="11" t="n"/>
-    </row>
-    <row r="8" ht="17.35" customHeight="1" s="8">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="B7" s="11" t="n"/>
+      <c r="C7" s="11" t="n"/>
+      <c r="D7" s="12" t="n"/>
+    </row>
+    <row r="8" ht="17.35" customHeight="1" s="9">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>Nota Fiscal</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A9" s="14" t="n"/>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="16" t="n">
+    <row r="9" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A9" s="15" t="n"/>
+      <c r="B9" s="15" t="n"/>
+      <c r="C9" s="16" t="n"/>
+      <c r="D9" s="17" t="n">
         <v>321.23</v>
       </c>
     </row>
-    <row r="10" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A10" s="14" t="n"/>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="16" t="n">
+    <row r="10" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A10" s="15" t="n"/>
+      <c r="B10" s="15" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="17" t="n">
         <v>21.4</v>
       </c>
     </row>
-    <row r="11" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A11" s="14" t="n"/>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="16" t="n">
+    <row r="11" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A11" s="15" t="n"/>
+      <c r="B11" s="15" t="n"/>
+      <c r="C11" s="16" t="n"/>
+      <c r="D11" s="17" t="n">
         <v>32.6</v>
       </c>
     </row>
-    <row r="12" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A12" s="17" t="inlineStr">
+    <row r="12" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n"/>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="14">
+      <c r="B12" s="19" t="n"/>
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="15">
         <f>sum(D9:D11)</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A13" s="19" t="n"/>
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-    </row>
-    <row r="14" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="13" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A13" s="20" t="n"/>
+      <c r="B13" s="20" t="n"/>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="20" t="n"/>
+    </row>
+    <row r="14" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Descricão Do Adiantamento</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n"/>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
-    </row>
-    <row r="15" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A15" s="17" t="inlineStr">
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+    </row>
+    <row r="15" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>Descrição</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B15" s="18" t="inlineStr">
         <is>
           <t>Data</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C15" s="18" t="inlineStr">
         <is>
           <t>Comprovante</t>
         </is>
       </c>
-      <c r="D15" s="17" t="inlineStr">
+      <c r="D15" s="18" t="inlineStr">
         <is>
           <t>Valor</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A16" s="19" t="n"/>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="19" t="n"/>
-      <c r="D16" s="19" t="n"/>
-    </row>
-    <row r="17" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A17" s="17" t="inlineStr">
+    <row r="16" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A16" s="20" t="n"/>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="20" t="n"/>
+      <c r="D16" s="20" t="n"/>
+    </row>
+    <row r="17" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>Receber</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n"/>
-      <c r="C17" s="17" t="inlineStr">
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>Devolver</t>
         </is>
       </c>
-      <c r="D17" s="18" t="n"/>
-    </row>
-    <row r="18" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A18" s="16">
+      <c r="D17" s="19" t="n"/>
+    </row>
+    <row r="18" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A18" s="17">
         <f>if(sum(D16:D15) - D12 &lt;0, D12 - sum(D16:D15), 0)</f>
         <v/>
       </c>
-      <c r="B18" s="18" t="n"/>
-      <c r="C18" s="16">
+      <c r="B18" s="19" t="n"/>
+      <c r="C18" s="17">
         <f>if(sum(D16:D15) - D12&lt;0, 0, sum(D16:D15) -  D12)</f>
         <v/>
       </c>
-      <c r="D18" s="18" t="n"/>
-    </row>
-    <row r="19" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A19" s="19" t="n"/>
-      <c r="B19" s="19" t="n"/>
-      <c r="C19" s="19" t="n"/>
-      <c r="D19" s="19" t="n"/>
-    </row>
-    <row r="20" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Apucarana, 24 de novembro de 2025 </t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="17.35" customFormat="1" customHeight="1" s="6">
-      <c r="A21" s="19" t="n"/>
-      <c r="B21" s="19" t="n"/>
-      <c r="C21" s="19" t="n"/>
-      <c r="D21" s="19" t="n"/>
-    </row>
-    <row r="22" ht="17.35" customHeight="1" s="8">
-      <c r="A22" s="19" t="inlineStr">
+      <c r="D18" s="19" t="n"/>
+    </row>
+    <row r="19" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A19" s="20" t="n"/>
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="20" t="n"/>
+      <c r="D19" s="20" t="n"/>
+    </row>
+    <row r="20" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apucarana, 08 de dezembro de 2025 </t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17.35" customFormat="1" customHeight="1" s="7">
+      <c r="A21" s="20" t="n"/>
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="20" t="n"/>
+      <c r="D21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="17.35" customHeight="1" s="9">
+      <c r="A22" s="20" t="inlineStr">
         <is>
           <t>__________________________________</t>
         </is>
       </c>
-      <c r="C22" s="19" t="inlineStr">
+      <c r="C22" s="20" t="inlineStr">
         <is>
           <t>__________________________________</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="17.35" customHeight="1" s="8">
-      <c r="A23" s="19" t="n"/>
-      <c r="C23" s="19" t="n"/>
-    </row>
-    <row r="24" ht="17.35" customHeight="1" s="8">
-      <c r="A24" s="19" t="n"/>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="19" t="n"/>
-      <c r="D24" s="19" t="n"/>
-    </row>
-    <row r="25" ht="17.35" customHeight="1" s="8">
-      <c r="A25" s="19" t="n"/>
-      <c r="B25" s="19" t="n"/>
-      <c r="C25" s="19" t="n"/>
-      <c r="D25" s="19" t="n"/>
-    </row>
-    <row r="26" ht="17.35" customHeight="1" s="8">
-      <c r="A26" s="19" t="n"/>
-      <c r="B26" s="19" t="n"/>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-    </row>
-    <row r="27" ht="17.35" customHeight="1" s="8">
-      <c r="A27" s="19" t="n"/>
-      <c r="B27" s="19" t="n"/>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-    </row>
-    <row r="28" ht="17.35" customHeight="1" s="8">
-      <c r="A28" s="19" t="n"/>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="19" t="n"/>
-      <c r="D28" s="19" t="n"/>
-    </row>
-    <row r="29" ht="17.35" customHeight="1" s="8">
-      <c r="A29" s="19" t="n"/>
-      <c r="B29" s="19" t="n"/>
-      <c r="C29" s="19" t="n"/>
-      <c r="D29" s="19" t="n"/>
-    </row>
-    <row r="30" ht="17.35" customHeight="1" s="8">
-      <c r="A30" s="19" t="n"/>
-      <c r="B30" s="19" t="n"/>
-      <c r="C30" s="19" t="n"/>
-      <c r="D30" s="19" t="n"/>
-    </row>
-    <row r="31" ht="17.35" customHeight="1" s="8">
-      <c r="A31" s="19" t="n"/>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="19" t="n"/>
-      <c r="D31" s="19" t="n"/>
-    </row>
-    <row r="32" ht="17.35" customHeight="1" s="8">
-      <c r="A32" s="19" t="n"/>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="19" t="n"/>
-      <c r="D32" s="19" t="n"/>
-    </row>
-    <row r="33" ht="17.35" customHeight="1" s="8">
-      <c r="A33" s="19" t="n"/>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="19" t="n"/>
-      <c r="D33" s="19" t="n"/>
-    </row>
-    <row r="34" ht="17.35" customHeight="1" s="8">
-      <c r="A34" s="19" t="n"/>
-      <c r="B34" s="19" t="n"/>
-      <c r="C34" s="19" t="n"/>
-      <c r="D34" s="19" t="n"/>
-    </row>
-    <row r="35" ht="17.35" customHeight="1" s="8">
-      <c r="A35" s="19" t="n"/>
-      <c r="B35" s="19" t="n"/>
-      <c r="C35" s="19" t="n"/>
-      <c r="D35" s="19" t="n"/>
-    </row>
-    <row r="36" ht="17.35" customHeight="1" s="8">
-      <c r="A36" s="19" t="n"/>
-      <c r="B36" s="19" t="n"/>
-      <c r="C36" s="19" t="n"/>
-      <c r="D36" s="19" t="n"/>
+    <row r="23" ht="17.35" customHeight="1" s="9">
+      <c r="A23" s="20" t="n"/>
+      <c r="C23" s="20" t="n"/>
+    </row>
+    <row r="24" ht="17.35" customHeight="1" s="9">
+      <c r="A24" s="20" t="n"/>
+      <c r="B24" s="20" t="n"/>
+      <c r="C24" s="20" t="n"/>
+      <c r="D24" s="20" t="n"/>
+    </row>
+    <row r="25" ht="17.35" customHeight="1" s="9">
+      <c r="A25" s="20" t="n"/>
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="20" t="n"/>
+      <c r="D25" s="20" t="n"/>
+    </row>
+    <row r="26" ht="17.35" customHeight="1" s="9">
+      <c r="A26" s="20" t="n"/>
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+    </row>
+    <row r="27" ht="17.35" customHeight="1" s="9">
+      <c r="A27" s="20" t="n"/>
+      <c r="B27" s="20" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+    </row>
+    <row r="28" ht="17.35" customHeight="1" s="9">
+      <c r="A28" s="20" t="n"/>
+      <c r="B28" s="20" t="n"/>
+      <c r="C28" s="20" t="n"/>
+      <c r="D28" s="20" t="n"/>
+    </row>
+    <row r="29" ht="17.35" customHeight="1" s="9">
+      <c r="A29" s="20" t="n"/>
+      <c r="B29" s="20" t="n"/>
+      <c r="C29" s="20" t="n"/>
+      <c r="D29" s="20" t="n"/>
+    </row>
+    <row r="30" ht="17.35" customHeight="1" s="9">
+      <c r="A30" s="20" t="n"/>
+      <c r="B30" s="20" t="n"/>
+      <c r="C30" s="20" t="n"/>
+      <c r="D30" s="20" t="n"/>
+    </row>
+    <row r="31" ht="17.35" customHeight="1" s="9">
+      <c r="A31" s="20" t="n"/>
+      <c r="B31" s="20" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="20" t="n"/>
+    </row>
+    <row r="32" ht="17.35" customHeight="1" s="9">
+      <c r="A32" s="20" t="n"/>
+      <c r="B32" s="20" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="20" t="n"/>
+    </row>
+    <row r="33" ht="17.35" customHeight="1" s="9">
+      <c r="A33" s="20" t="n"/>
+      <c r="B33" s="20" t="n"/>
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="20" t="n"/>
+    </row>
+    <row r="34" ht="17.35" customHeight="1" s="9">
+      <c r="A34" s="20" t="n"/>
+      <c r="B34" s="20" t="n"/>
+      <c r="C34" s="20" t="n"/>
+      <c r="D34" s="20" t="n"/>
+    </row>
+    <row r="35" ht="17.35" customHeight="1" s="9">
+      <c r="A35" s="20" t="n"/>
+      <c r="B35" s="20" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="20" t="n"/>
+    </row>
+    <row r="36" ht="17.35" customHeight="1" s="9">
+      <c r="A36" s="20" t="n"/>
+      <c r="B36" s="20" t="n"/>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="19">

</xml_diff>